<commit_message>
Matrice mise à jour automatiquement (22/10/2026 18:17)
</commit_message>
<xml_diff>
--- a/matrices/MATRICE_DE_SUIVI_DES_ACTIVITES_du_22-10-26.xlsx
+++ b/matrices/MATRICE_DE_SUIVI_DES_ACTIVITES_du_22-10-26.xlsx
@@ -15,8 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0\ &quot;CFA&quot;"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -208,7 +209,7 @@
     <xf numFmtId="9" fontId="9" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -373,6 +374,7 @@
     <xf numFmtId="164" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -482,7 +484,7 @@
     <from>
       <col>22</col>
       <colOff>38100</colOff>
-      <row>5</row>
+      <row>4</row>
       <rowOff>38100</rowOff>
     </from>
     <ext cx="1066800" cy="800100"/>
@@ -493,6 +495,56 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>22</col>
+      <colOff>38100</colOff>
+      <row>5</row>
+      <rowOff>38100</rowOff>
+    </from>
+    <ext cx="1066800" cy="800100"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>22</col>
+      <colOff>38100</colOff>
+      <row>6</row>
+      <rowOff>38100</rowOff>
+    </from>
+    <ext cx="1066800" cy="800100"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1002,16 +1054,16 @@
         <v>100</v>
       </c>
       <c r="Q4" s="25" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R4" s="26" t="inlineStr">
         <is>
-          <t>Non démarré</t>
+          <t>Travaux achevés</t>
         </is>
       </c>
       <c r="S4" s="21" t="inlineStr">
         <is>
-          <t>Non transmis</t>
+          <t>Transmis en cours de validation</t>
         </is>
       </c>
       <c r="T4" s="21" t="inlineStr">
@@ -1019,12 +1071,16 @@
           <t>AGIR</t>
         </is>
       </c>
-      <c r="U4" s="27" t="n"/>
-      <c r="V4" s="27" t="n"/>
+      <c r="U4" s="64" t="n">
+        <v>46289</v>
+      </c>
+      <c r="V4" s="64" t="n">
+        <v>46317</v>
+      </c>
       <c r="W4" s="27" t="n"/>
       <c r="X4" s="21" t="inlineStr">
         <is>
-          <t>Emmanuel aka - PCR</t>
+          <t>Kouadio - Pcr</t>
         </is>
       </c>
       <c r="Y4" s="11" t="n"/>
@@ -1098,11 +1154,11 @@
       <c r="O5" s="22" t="n"/>
       <c r="P5" s="22" t="n"/>
       <c r="Q5" s="25" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="R5" s="26" t="inlineStr">
         <is>
-          <t>Demarrage autorisé</t>
+          <t>Travaux en cours</t>
         </is>
       </c>
       <c r="S5" s="21" t="inlineStr">
@@ -1112,13 +1168,17 @@
       </c>
       <c r="T5" s="21" t="inlineStr">
         <is>
-          <t>ONG EPC</t>
+          <t>RIDDEF</t>
         </is>
       </c>
       <c r="U5" s="27" t="n"/>
       <c r="V5" s="27" t="n"/>
       <c r="W5" s="27" t="n"/>
-      <c r="X5" s="28" t="n"/>
+      <c r="X5" s="21" t="inlineStr">
+        <is>
+          <t>Emmanuel AKA - Pcr Ci</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="75" customFormat="1" customHeight="1" s="2">
       <c r="B6" s="21" t="n">
@@ -1177,21 +1237,21 @@
       <c r="O6" s="52" t="n"/>
       <c r="P6" s="22" t="n"/>
       <c r="Q6" s="25" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="R6" s="26" t="inlineStr">
         <is>
-          <t>Non démarré</t>
+          <t>Travaux en cours</t>
         </is>
       </c>
       <c r="S6" s="21" t="inlineStr">
         <is>
-          <t>Non transmis</t>
+          <t>Validé</t>
         </is>
       </c>
       <c r="T6" s="21" t="inlineStr">
         <is>
-          <t>AGIR pour ODD</t>
+          <t>Non mobilisée</t>
         </is>
       </c>
       <c r="U6" s="27" t="n"/>
@@ -1199,7 +1259,7 @@
       <c r="W6" s="27" t="n"/>
       <c r="X6" s="21" t="inlineStr">
         <is>
-          <t>Ev - PCR</t>
+          <t>Kouadio - Pcr</t>
         </is>
       </c>
     </row>
@@ -1257,23 +1317,27 @@
       </c>
       <c r="R7" s="26" t="inlineStr">
         <is>
-          <t>Demarrage autorisé</t>
+          <t>Non démarré – Retard</t>
         </is>
       </c>
       <c r="S7" s="21" t="inlineStr">
         <is>
-          <t>Transmis</t>
+          <t>Non transmis</t>
         </is>
       </c>
       <c r="T7" s="21" t="inlineStr">
         <is>
-          <t>AGIR pour ODD</t>
+          <t>Non mobilisée</t>
         </is>
       </c>
       <c r="U7" s="27" t="n"/>
       <c r="V7" s="27" t="n"/>
       <c r="W7" s="27" t="n"/>
-      <c r="X7" s="28" t="n"/>
+      <c r="X7" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emmanuel AKA - Pcr </t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="60" customFormat="1" customHeight="1" s="3">
       <c r="B8" s="30" t="n">

</xml_diff>

<commit_message>
Matrice mise à jour automatiquement (22/10/2026 18:34)
</commit_message>
<xml_diff>
--- a/matrices/MATRICE_DE_SUIVI_DES_ACTIVITES_du_22-10-26.xlsx
+++ b/matrices/MATRICE_DE_SUIVI_DES_ACTIVITES_du_22-10-26.xlsx
@@ -1054,21 +1054,21 @@
         <v>100</v>
       </c>
       <c r="Q4" s="25" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="R4" s="26" t="inlineStr">
         <is>
-          <t>Travaux achevés</t>
+          <t>Non démarré</t>
         </is>
       </c>
       <c r="S4" s="21" t="inlineStr">
         <is>
-          <t>Transmis en cours de validation</t>
+          <t>Non transmis</t>
         </is>
       </c>
       <c r="T4" s="21" t="inlineStr">
         <is>
-          <t>AGIR</t>
+          <t>Non mobilisée</t>
         </is>
       </c>
       <c r="U4" s="64" t="n">
@@ -1154,7 +1154,7 @@
       <c r="O5" s="22" t="n"/>
       <c r="P5" s="22" t="n"/>
       <c r="Q5" s="25" t="n">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="R5" s="26" t="inlineStr">
         <is>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="T5" s="21" t="inlineStr">
         <is>
-          <t>RIDDEF</t>
+          <t>ASAPSU</t>
         </is>
       </c>
       <c r="U5" s="27" t="n"/>
@@ -1176,7 +1176,7 @@
       <c r="W5" s="27" t="n"/>
       <c r="X5" s="21" t="inlineStr">
         <is>
-          <t>Emmanuel AKA - Pcr Ci</t>
+          <t>Kouadio</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1237,7 @@
       <c r="O6" s="52" t="n"/>
       <c r="P6" s="22" t="n"/>
       <c r="Q6" s="25" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="R6" s="26" t="inlineStr">
         <is>
@@ -1259,7 +1259,7 @@
       <c r="W6" s="27" t="n"/>
       <c r="X6" s="21" t="inlineStr">
         <is>
-          <t>Kouadio - Pcr</t>
+          <t xml:space="preserve">Emmanuel A - Pcr </t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,9 @@
 KANTARA</t>
         </is>
       </c>
-      <c r="K7" s="22" t="n"/>
+      <c r="K7" s="52" t="n">
+        <v>46320</v>
+      </c>
       <c r="L7" s="22" t="n">
         <v>4</v>
       </c>
@@ -1313,21 +1315,21 @@
       <c r="O7" s="22" t="n"/>
       <c r="P7" s="22" t="n"/>
       <c r="Q7" s="25" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="R7" s="26" t="inlineStr">
         <is>
-          <t>Non démarré – Retard</t>
+          <t>Travaux suspendus</t>
         </is>
       </c>
       <c r="S7" s="21" t="inlineStr">
         <is>
-          <t>Non transmis</t>
+          <t>Validé</t>
         </is>
       </c>
       <c r="T7" s="21" t="inlineStr">
         <is>
-          <t>Non mobilisée</t>
+          <t>RIDDEF</t>
         </is>
       </c>
       <c r="U7" s="27" t="n"/>
@@ -1335,7 +1337,7 @@
       <c r="W7" s="27" t="n"/>
       <c r="X7" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emmanuel AKA - Pcr </t>
+          <t>Emmanuel - Pcr</t>
         </is>
       </c>
     </row>

</xml_diff>